<commit_message>
data: Update configuration tables and regenerate DataTable classes
- Regenerate SummonChessTable.cs from updated Excel data
- Update BuffTable, CardTable, EnemyEntityTable configurations
- Update ResourceConfigTable with new resource IDs
- Sync .csproj files with latest assembly references
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/SummonChessSkillTable.xlsx
+++ b/AAAGameData/DataTables/SummonChessSkillTable.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="118">
   <si>
     <t>#</t>
   </si>
@@ -284,7 +284,7 @@
     <t>邪灵被动：普攻命中30%概率对目标施加恐惧（攻击力-20%，持续2s）</t>
   </si>
   <si>
-    <t>邪灵爪击</t>
+    <t>邪灵普攻</t>
   </si>
   <si>
     <t>邪灵普攻：近战物理伤害</t>
@@ -305,7 +305,82 @@
     <t>{"MagicCircleId":3009,"SpawnHeight":0.1,"DotInterval":1,"CorrosionInterval":5,"DotDamageCoeff":0.25,"DotBaseDamage":10,"ExplosionDamageCoeff":1.2,"ExplosionBaseDamage":30}</t>
   </si>
   <si>
-    <t>邪灵技能二：锁定目标位置生成法阵；敌人首次进入立即获得2层腐蚀；法阵内持续受到魔法伤害且每停留5秒叠加1层腐蚀（离开重置）；爆炸时对范围内敌人造成大量伤害并再施加1层腐蚀</t>
+    <t>邪灵大招：锁定目标位置生成法阵；敌人首次进入立即获得2层腐蚀；法阵内持续受到魔法伤害且每停留5秒叠加1层腐蚀（离开重置）；爆炸时对范围内敌人造成大量伤害并再施加1层腐蚀</t>
+  </si>
+  <si>
+    <t>虚无之躯</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>恶魂被动：物理伤害减免30%，虚无之物难以被伤害</t>
+  </si>
+  <si>
+    <t>恶魂普攻</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>恶魂普攻：发射黑暗能量球造成法术伤害，20%概率使目标陷入恐惧</t>
+  </si>
+  <si>
+    <t>心灵扭曲</t>
+  </si>
+  <si>
+    <t>5009</t>
+  </si>
+  <si>
+    <t>恶魂技能一：诵读古老音节，对范围内敌人造成法术伤害，使其陷入混乱状态</t>
+  </si>
+  <si>
+    <t>邪念潮涌</t>
+  </si>
+  <si>
+    <t>5009,9</t>
+  </si>
+  <si>
+    <t>恶魂大招：释放压抑已久的邪念怨恨发出冲击，对前方范围内所有敌人造成法术伤害，施加混乱状态并60%概率造成恐惧</t>
+  </si>
+  <si>
+    <t>黑暗神力</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>黑暗杨戬被动：所有攻击附带腐蚀效果，多阶段Boss</t>
+  </si>
+  <si>
+    <t>黑暗戟横扫</t>
+  </si>
+  <si>
+    <t>黑暗杨戬普攻：以黑暗戟横扫，造成物理伤害</t>
+  </si>
+  <si>
+    <t>天威圣戟·黑暗</t>
+  </si>
+  <si>
+    <t>黑暗杨戬技能一：范围清盾技能</t>
+  </si>
+  <si>
+    <t>三眼天火</t>
+  </si>
+  <si>
+    <t>黑暗杨戬技能二：直线法术伤害，施加灼烧</t>
+  </si>
+  <si>
+    <t>堕落劈山</t>
+  </si>
+  <si>
+    <t>黑暗杨戬大招：真实伤害，留下黑暗裂缝</t>
+  </si>
+  <si>
+    <t>撕咬</t>
+  </si>
+  <si>
+    <t>黑暗哮天犬普攻：近战物理伤害，附带流血</t>
   </si>
 </sst>
 </file>
@@ -1280,15 +1355,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="47" customWidth="1"/>
-    <col min="6" max="6" width="15.625" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="41" customWidth="1"/>
     <col min="8" max="9" width="50" customWidth="1"/>
     <col min="10" max="10" width="41" customWidth="1"/>
@@ -1307,8 +1382,7 @@
     <col min="23" max="24" width="16" customWidth="1"/>
     <col min="25" max="25" width="20" customWidth="1"/>
     <col min="26" max="26" width="16" customWidth="1"/>
-    <col min="27" max="27" width="171.625" customWidth="1"/>
-    <col min="28" max="28" width="50" customWidth="1"/>
+    <col min="27" max="28" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">
@@ -2565,6 +2639,806 @@
         <v>92</v>
       </c>
     </row>
+    <row r="17" ht="15" customHeight="1" spans="1:28">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1">
+        <v>41</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>0</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="V17" s="1">
+        <v>0</v>
+      </c>
+      <c r="W17" s="1">
+        <v>1841</v>
+      </c>
+      <c r="X17" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="1"/>
+      <c r="AB17" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" spans="1:28">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1">
+        <v>42</v>
+      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="1">
+        <v>2</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>2</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="I18" s="1">
+        <v>2</v>
+      </c>
+      <c r="J18" s="1">
+        <v>3010</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="N18" s="1">
+        <v>20</v>
+      </c>
+      <c r="O18" s="1">
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>0</v>
+      </c>
+      <c r="R18" s="1">
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <v>1</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="U18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V18" s="1">
+        <v>15</v>
+      </c>
+      <c r="W18" s="1">
+        <v>1842</v>
+      </c>
+      <c r="X18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="1"/>
+      <c r="AB18" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" spans="1:28">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1">
+        <v>43</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="1">
+        <v>3</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" s="1">
+        <v>2</v>
+      </c>
+      <c r="H19" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="I19" s="1">
+        <v>3</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>1</v>
+      </c>
+      <c r="L19" s="1">
+        <v>40</v>
+      </c>
+      <c r="M19" s="1">
+        <v>50</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <v>9</v>
+      </c>
+      <c r="P19" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <v>1</v>
+      </c>
+      <c r="S19" s="1">
+        <v>0</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="U19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V19" s="1">
+        <v>0</v>
+      </c>
+      <c r="W19" s="1">
+        <v>1843</v>
+      </c>
+      <c r="X19" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="1"/>
+      <c r="AB19" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" spans="1:28">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1">
+        <v>44</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="1">
+        <v>4</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>2</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="I20" s="1">
+        <v>3</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>1</v>
+      </c>
+      <c r="L20" s="1">
+        <v>50</v>
+      </c>
+      <c r="M20" s="1">
+        <v>70</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1">
+        <v>15</v>
+      </c>
+      <c r="P20" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q20" s="1">
+        <v>0</v>
+      </c>
+      <c r="R20" s="1">
+        <v>1</v>
+      </c>
+      <c r="S20" s="1">
+        <v>0</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="U20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V20" s="1">
+        <v>0</v>
+      </c>
+      <c r="W20" s="1">
+        <v>1844</v>
+      </c>
+      <c r="X20" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:28">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1">
+        <v>51</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1">
+        <v>0</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
+        <v>0</v>
+      </c>
+      <c r="P21" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>0</v>
+      </c>
+      <c r="R21" s="1">
+        <v>0</v>
+      </c>
+      <c r="S21" s="1">
+        <v>0</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V21" s="1">
+        <v>0</v>
+      </c>
+      <c r="W21" s="1">
+        <v>1845</v>
+      </c>
+      <c r="X21" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="1"/>
+      <c r="AB21" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:28">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1">
+        <v>52</v>
+      </c>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="1">
+        <v>2</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0</v>
+      </c>
+      <c r="G22" s="1">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0</v>
+      </c>
+      <c r="K22" s="1">
+        <v>1</v>
+      </c>
+      <c r="L22" s="1">
+        <v>0</v>
+      </c>
+      <c r="M22" s="1">
+        <v>0</v>
+      </c>
+      <c r="N22" s="1">
+        <v>15</v>
+      </c>
+      <c r="O22" s="1">
+        <v>0</v>
+      </c>
+      <c r="P22" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>0</v>
+      </c>
+      <c r="R22" s="1">
+        <v>1</v>
+      </c>
+      <c r="S22" s="1">
+        <v>0</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="U22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V22" s="1">
+        <v>0</v>
+      </c>
+      <c r="W22" s="1">
+        <v>1846</v>
+      </c>
+      <c r="X22" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="1"/>
+      <c r="AB22" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" spans="1:28">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1">
+        <v>53</v>
+      </c>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" s="1">
+        <v>3</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="I23" s="1">
+        <v>3</v>
+      </c>
+      <c r="J23" s="1">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1">
+        <v>1</v>
+      </c>
+      <c r="L23" s="1">
+        <v>40</v>
+      </c>
+      <c r="M23" s="1">
+        <v>50</v>
+      </c>
+      <c r="N23" s="1">
+        <v>0</v>
+      </c>
+      <c r="O23" s="1">
+        <v>8</v>
+      </c>
+      <c r="P23" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>0</v>
+      </c>
+      <c r="R23" s="1">
+        <v>1</v>
+      </c>
+      <c r="S23" s="1">
+        <v>0</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="U23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V23" s="1">
+        <v>0</v>
+      </c>
+      <c r="W23" s="1">
+        <v>1847</v>
+      </c>
+      <c r="X23" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" spans="1:28">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1">
+        <v>54</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" s="1">
+        <v>3</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1">
+        <v>2</v>
+      </c>
+      <c r="H24" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="I24" s="1">
+        <v>2</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0</v>
+      </c>
+      <c r="K24" s="1">
+        <v>1</v>
+      </c>
+      <c r="L24" s="1">
+        <v>40</v>
+      </c>
+      <c r="M24" s="1">
+        <v>50</v>
+      </c>
+      <c r="N24" s="1">
+        <v>0</v>
+      </c>
+      <c r="O24" s="1">
+        <v>9</v>
+      </c>
+      <c r="P24" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>0</v>
+      </c>
+      <c r="R24" s="1">
+        <v>1</v>
+      </c>
+      <c r="S24" s="1">
+        <v>0</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V24" s="1">
+        <v>0</v>
+      </c>
+      <c r="W24" s="1">
+        <v>1848</v>
+      </c>
+      <c r="X24" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="1"/>
+      <c r="AB24" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" spans="1:28">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1">
+        <v>55</v>
+      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="1">
+        <v>4</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1">
+        <v>3</v>
+      </c>
+      <c r="H25" s="1">
+        <v>2</v>
+      </c>
+      <c r="I25" s="1">
+        <v>1</v>
+      </c>
+      <c r="J25" s="1">
+        <v>0</v>
+      </c>
+      <c r="K25" s="1">
+        <v>1</v>
+      </c>
+      <c r="L25" s="1">
+        <v>100</v>
+      </c>
+      <c r="M25" s="1">
+        <v>100</v>
+      </c>
+      <c r="N25" s="1">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1">
+        <v>15</v>
+      </c>
+      <c r="P25" s="1">
+        <v>8</v>
+      </c>
+      <c r="Q25" s="1">
+        <v>0</v>
+      </c>
+      <c r="R25" s="1">
+        <v>1</v>
+      </c>
+      <c r="S25" s="1">
+        <v>0</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="U25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V25" s="1">
+        <v>0</v>
+      </c>
+      <c r="W25" s="1">
+        <v>1849</v>
+      </c>
+      <c r="X25" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="1"/>
+      <c r="AB25" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" spans="1:28">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1">
+        <v>56</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E26" s="1">
+        <v>2</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1">
+        <v>1</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1</v>
+      </c>
+      <c r="J26" s="1">
+        <v>0</v>
+      </c>
+      <c r="K26" s="1">
+        <v>1</v>
+      </c>
+      <c r="L26" s="1">
+        <v>0</v>
+      </c>
+      <c r="M26" s="1">
+        <v>0</v>
+      </c>
+      <c r="N26" s="1">
+        <v>15</v>
+      </c>
+      <c r="O26" s="1">
+        <v>0</v>
+      </c>
+      <c r="P26" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="1">
+        <v>0</v>
+      </c>
+      <c r="R26" s="1">
+        <v>1</v>
+      </c>
+      <c r="S26" s="1">
+        <v>0</v>
+      </c>
+      <c r="T26" s="2">
+        <v>23</v>
+      </c>
+      <c r="U26" s="2">
+        <v>0</v>
+      </c>
+      <c r="V26" s="1">
+        <v>0</v>
+      </c>
+      <c r="W26" s="1">
+        <v>1850</v>
+      </c>
+      <c r="X26" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>